<commit_message>
docs(qa): update Avanzamento progress sheet with QA findings
Re-grade 14 rows after the QA pass: 9 red items were actually implemented
(now yellow/green), account naming resolved, forecast/period-comparison
verified. Net: 0 red (was 9). Notes prefixed [QA 01/06/2026].

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Avanzamento tool Niuexa.xlsx
+++ b/Avanzamento tool Niuexa.xlsx
@@ -547,12 +547,12 @@
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Da preview non è ancora presente</t>
+          <t>[QA 01/06/2026] Endpoint GET /reports/inventory + export CSV implementati e funzionanti (storico snapshot + low_stock). Nessun dato nell'org di test (i 5 record sono in altro org). Da verificare con sync SP-API reale.</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>Da migliorare; da preview non venivano restituiti i dati</t>
+          <t>[QA 01/06/2026] competitors=0 nel seed. La discovery usa SP-API catalog search (NON Helium10): 0 risultati con credenziali attuali -&gt; richiede SP-API valido. Il fallimento per-ASIN non rompe il report (verificato).</t>
         </is>
       </c>
     </row>
@@ -678,12 +678,12 @@
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>Da preview non è ancora presente</t>
+          <t>[QA 01/06/2026] GET /reports/orders implementato (filtri account/periodo, validazione date OK). 3 ordini presenti ma in altro org. Da verificare con dati reali.</t>
         </is>
       </c>
     </row>
@@ -705,12 +705,12 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>Da preview non è ancora presente</t>
+          <t>[QA 01/06/2026] Migration 023 partiziona sales_data/advertising_metrics/advertising_metrics_by_asin/bsr_history per mese (+ bootstrap 24 mesi). Corretto bug di 'alembic upgrade head' (sequence ownership + ripristinate funzioni della migration 015). Nessuna perdita dati.</t>
         </is>
       </c>
     </row>
@@ -732,12 +732,12 @@
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>Da preview, non presente il confronto immediato</t>
+          <t>[QA 01/06/2026] Confronto periodo-su-periodo verificato in dashboard (previous_value + % change corretti, no NaN/Inf). MoM OK; YoY = stesso meccanismo su range annuale.</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>Da migliorare; da preview non venivano restituiti i dati</t>
+          <t>[QA 01/06/2026] Dipende dai dati competitor (vedi riga 10). Comparison-matrix gestita (400 chiaro se nessun competitor). Da sbloccare con SP-API valido.</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>Da preview non è ancora presente</t>
+          <t>[QA 01/06/2026] GET /analytics/returns implementato con stato vuoto gestito graziosamente (no crash, divisione per zero protetta). returns_data=0 nel seed: da verificare con dati resi reali.</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>Da preview non è ancora integrata funzionalità</t>
+          <t>[QA 01/06/2026] POST /catalog/bulk-update + template scaricabile + validazione file implementati e funzionanti (file invalido -&gt; 400 chiaro). Push reale ad Amazon richiede credenziali SP-API con permessi di scrittura (Seller).</t>
         </is>
       </c>
     </row>
@@ -971,12 +971,12 @@
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>Da preview non è ancora integrata funzionalità</t>
+          <t>[QA 01/06/2026] POST /catalog/prices implementato con validazione (prezzo negativo/decimali extra -&gt; 422). Scrittura reale richiede SP-API write (Seller Central).</t>
         </is>
       </c>
     </row>
@@ -998,12 +998,12 @@
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>Da preview non è ancora integrata funzionalità</t>
+          <t>[QA 01/06/2026] PATCH /catalog/products/{asin}/availability implementato; corretto bug 500 su errori SP-API non-throttle (ora 4xx chiaro). Scrittura reale richiede SP-API write.</t>
         </is>
       </c>
     </row>
@@ -1025,12 +1025,12 @@
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>Da preview non è ancora integrata funzionalità</t>
+          <t>[QA 01/06/2026] Endpoint immagini (POST/GET/DELETE) + validazione tipo (JPG/PNG accettati, file non validi rifiutati) implementati. Upload reale richiede credenziali AWS S3/R2.</t>
         </is>
       </c>
     </row>
@@ -1052,12 +1052,12 @@
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>Modello Prophet + horizon caps + MAPE/RMSE/confidence già presenti. Chiariti labels: la previsione è di fatturato (revenue), non unità; rinominate colonna "Predicted total (revenue)" e label export "Sales Forecast (revenue)". available-products ora restituisce ASIN non idonei con is_eligible/reason, invece di nasconderli silenziosamente. Resta da estendere a forecast unità esplicito se richiesto.</t>
+          <t>[QA 01/06/2026] Prophet + horizon caps (30/60/90) + MAPE/RMSE/confidence + label IT chiarite (no overpromise). Tutti i 44 ASIN selezionabili (quelli con poco storico mostrati disabilitati con motivo). Verificato.</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>Da preview non è ancora presente</t>
+          <t>[QA 01/06/2026] GET /analytics/product-trends implementato e risponde (insight su storico insufficiente con dati attuali). Da arricchire con piu' storico.</t>
         </is>
       </c>
     </row>
@@ -1202,12 +1202,12 @@
       </c>
       <c r="D31" s="14" t="inlineStr">
         <is>
-          <t>🟡</t>
-        </is>
-      </c>
-      <c r="E31" s="17" t="inlineStr">
-        <is>
-          <t>UI Accounts evidenzia i nomi segnaposto con badge + banner; rinomina via PUT /api/v1/accounts/{id} o via script backend/scripts/rename_amazon_account.py. Bloccato dai nomi-cliente reali da fornire.</t>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>[QA 01/06/2026] RISOLTO: account rinominati (real-&gt;Bitron, second account-&gt;Dialcos) via PUT /api/v1/accounts/{id}; persistenza verificata (refresh + re-login). UI evidenzia segnaposto con badge/banner di rinomina.</t>
         </is>
       </c>
     </row>

</xml_diff>